<commit_message>
Add 35 coded competition entries and write_entries.py
Hand-coded 35 top-finishing Kaggle competition solutions (Playground Series S3-S5
and Featured competitions) into kaggle_meta_analysis.xlsx with all schema fields:
preprocessing decisions, feature engineering techniques, model choices, CV strategy,
ensemble methods, and writeup metadata.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kaggle_meta_analysis.xlsx
+++ b/data/kaggle_meta_analysis.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AB36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -611,6 +611,4256 @@
       <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>original_data_usage</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>icr-identify-age-related-conditions</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ICR - Identifying Age-Related Conditions</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Featured</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>6430</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2023-08-14</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>56</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>No FE (overfitting); multi-label CV strategy; reweighting probabilities at output</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>playground-series-s4e7</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Binary Classification of Insurance Cross Selling</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2234</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2024-07-31</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>stratified_kfold</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Feature store (12 versions); component models on feature subsets (previously insured, vehicle damage); feature importance via CatBoost single-fold</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, NN</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>CatBoost</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>playground-series-s5e3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Binary Prediction with a Rainfall Dataset</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>4381</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>grouped</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>blending</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>No FE; original data added as new columns via target mapping (merge_columns approach)</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>XGBoost, CatBoost, TabPFN, LogisticRegression, SVC, SVR</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>SVC</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>merge_columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>playground-series-s5e5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Predict Calorie Expenditure</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4316</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2025-05-31</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>hill_climbing</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>log1p transforms; product/division/sum/diff pairs; binned features (9 bins); groupby z-score features (26); residual modeling (NN on LR residuals, XGB on NN residuals); cuML TargetEncoder</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>XGBoost, CatBoost, NN, LinearRegression</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>playground-series-s5e12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Diabetes Prediction Challenge</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4206</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>post_cutoff</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Rank transformation; varied FE approaches across ~100 base models</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, NN, Ridge, AutoML</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>playground-series-s5e10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Predicting Road Accident Risk</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>4082</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2025-10-31</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Autoencoder latent features; genetic programming features (11 GP); XGBoost residual boosting; multiple feature type representations (categorical/numerical/mixed)</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>XGBoost, CatBoost, NN, Lasso, AutoGluon, Autoencoder</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Loan Approval Prediction</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3858</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2024-10-31</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Dual numeric+categorical feature representation; large max_bin values; original dataset included</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>LightGBM, XGBoost, CatBoost, NN</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>CatBoost</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>optuna</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>playground-series-s5e11</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Predicting Loan Payback</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>3724</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>hill_climbing</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Digit extraction from numericals; pairwise/triple/quadruple digit interactions + TE/CE; base feature pairs + TE/CE; quantile binning; categorical version of credit_score; TE with alternative targets</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, NN, LogisticRegression, RandomForest, ExtraTrees</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>playground-series-s4e1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Binary Classification with a Bank Churn Dataset</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3632</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2024-01-31</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="n">
+        <v>2</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>blending</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Subset matching — all 1-10 element feature subsets checked against original dataset (~1000 binary indicators); CustomerId+Surname subset; post-processing probability shift</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>LightGBM, AutoGluon</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>AutoGluon</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>feature_lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>playground-series-s5e2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Backpack Prediction Challenge</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3393</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="n">
+        <v>3</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>ordinal</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>Groupby aggregations (mean/std/count/min/max/nunique/skew); groupby histogram bins; groupby quantiles; NaN base-2 encoding; numerical rounding/binning; digit extraction from floats; categorical column combinations (all pairs); division features (ratios of aggregated features)</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>merge_columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>playground-series-s5e8</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Binary Classification with a Bank Dataset</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>3365</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" t="n">
+        <v>2</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>TE/CE on feature bigrams (competition + original targets); products of numerical bigrams; cyclical features</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, NN, RandomForest</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>playground-series-s5e4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Predict Podcast Listening Time</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>3310</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2025-04-30</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>3</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>Target ratio transformation (target/Episode_Length); Episode_Length imputation via model; pseudo labeling (train+test); residual boosting (GBDT on Lasso/SVR/MLP residuals); 6000 features for linear models; diverse feature sets per model</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, NN, Lasso, SVR, KNN, RandomForest, AutoGluon</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>playground-series-s4e9</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Regression of Used Car Prices</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>3066</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>3</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>clip</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>CatBoost classifier OOF as feature for LGBM; SVR OOF as NN feature; median target encoding (leakfree per fold); rare category grouping; outlier price binning via IQR</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>LightGBM, CatBoost, SVR, NN, XGBoost, AutoGluon</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>optuna</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e5</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Regression with a Flood Prediction Dataset</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2788</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2024-05-31</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Row-wise statistics (sum/std/max); sorted features; count threshold features (nb_sup6/7/8); target encoding on row sum; target transformation (subtract feature mean x0.1); permutation + backward feature selection</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, AutoGluon</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>optuna</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>playground-series-s4e11</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Exploring Mental Health Data</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2685</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2024-11-30</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" t="n">
+        <v>2</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, AutoGluon</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>AutoGluon</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>playground-series-s5e6</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Predicting Optimal Fertilizers</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2648</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>multiclass</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>stratified_kfold</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>hill_climbing</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>All pairs/triples/quadruples of 8 features (162 combos); TE of 162 combos x7 binary targets (2268 cols); TE using original dataset; residual boosting (XGB over LR base margin); pseudo labeling; repeated KFold seed averaging; retrain on 100% data</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, NN, LinearRegression, KNN</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>concat_rows, merge_columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>playground-series-s4e8</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Binary Prediction of Poisonous Mushrooms</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>2422</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2024-08-31</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" t="n">
+        <v>2</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>Original dataset poisonous probability as engineered feature; confident disagreement overwriting (predictions &gt;0.99 threshold)</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>LightGBM, XGBoost, CatBoost, RandomForest, ExtraTrees, AutoGluon</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>playground-series-s4e12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Regression with an Insurance Dataset</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>2390</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" t="n">
+        <v>3</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Label encoding; TE (mean/median/min/max/nunique) + CE per column; column combinations (2-6 way); treating numerics as categorical + TE/CE; Policy Start Date decomposition; GPU-accelerated search of 145K+ combinations -&gt; 170 kept</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>playground-series-s4e3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Steel Plate Defect Prediction</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2199</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2024-03-31</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>multiclass</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" t="n">
+        <v>3</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>drop</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>blending</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>Ratio features (length/thickness); range x area interaction; min-max normalized thickness feature; feature dropping via CV + feature importance + correlation</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, HistGB</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>optuna</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>playground-series-s3e24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Binary Prediction of Smoker Status using Bio-Signals</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1908</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2023-12-31</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>3</v>
+      </c>
+      <c r="N21" t="n">
+        <v>2</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>stratified_kfold</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>blending</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>Brute-force feature combinations (80-120 kept); permutation importance for feature pruning</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>LightGBM, XGBoost, CatBoost, RandomForest, LogisticRegression, TabNet, NN, GAM</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>optuna</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>playground-series-s3e23</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Binary Classification with a Software Defects Dataset</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1702</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2023-11-30</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M22" t="n">
+        <v>2</v>
+      </c>
+      <c r="N22" t="n">
+        <v>3</v>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>hill_climbing</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>Log transformation of all features (core improvement); PCA/t-SNE/clustering tried but failed</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>LightGBM, XGBoost, CatBoost, RandomForest, ExtraTrees, HistGB, LogisticRegression, NN</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>playground-series-s3e14</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Regression with a Wild Blueberry Yield Dataset</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1875</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2023-07-31</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" t="n">
+        <v>2</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>Post-processing: match test rows to original dataset by fruitset+fruitmass key -&gt; assign original yield values; automated matching script (2073 test samples x 776 unique yields)</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>feature_lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>playground-series-s3e26</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Multi-Class Prediction of Cirrhosis Outcomes</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1661</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>multiclass</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>2</v>
+      </c>
+      <c r="N24" t="n">
+        <v>2</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OHE</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>Piecewise linear encoding (PLE) for continuous features; embedding layers for categorical features (edema, stage)</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, NN</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>optuna</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>playground-series-s3e16</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Regression with a Crab Age Dataset</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1429</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2023-08-31</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>3</v>
+      </c>
+      <c r="N25" t="n">
+        <v>2</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>stratified_kfold</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>Domain features (meat yield/surface area/weight ratios/pseudo BMI/viscera ratio); log transform on weight; post-processing (round to nearest integer); feature subset selection (6-10 features per model)</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, HistGB</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>optuna</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>playground-series-s3e17</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Binary Classification of Machine Failures</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1502</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2023-09-30</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>3</v>
+      </c>
+      <c r="N26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>None described — AutoML handles internally</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>AutoML</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>playground-series-s3e11</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Regression with a Tabular Media Campaign Cost Dataset</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>952</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2023-06-15</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>1</v>
+      </c>
+      <c r="N27" t="n">
+        <v>3</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>blending</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>Feature subset selection across models; duplicate grouping (360K-&gt;3000 groups); log1p target transformation; store_sqft treated as categorical</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>LightGBM, XGBoost, CatBoost, RandomForest, ExtraTrees, NN</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>playground-series-s3e13</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Classification with a Tabular Vector Borne Disease Dataset</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>934</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2023-07-15</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>multiclass</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>1</v>
+      </c>
+      <c r="N28" t="n">
+        <v>1</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>blending</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>LightGBM, NN, Autoencoder</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>playground-series-s3e5</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Ordinal Regression with a Tabular Wine Quality Dataset</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>901</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2023-03-31</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>multiclass</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>1</v>
+      </c>
+      <c r="N29" t="n">
+        <v>2</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>stratified_kfold</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>None — FE tried but worsened CV; post-processing with OptimizedRounder for ordinal class cutoffs</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>optuna</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>not_used</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>playground-series-s3e10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Binary Classification with a Tabular Pulsar Dataset</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>807</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2023-05-31</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M30" t="n">
+        <v>1</v>
+      </c>
+      <c r="N30" t="n">
+        <v>2</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>XGBoost predictions as GAM input features; Lasso predictions as GAM input features; interaction terms in GAM</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>GAM, XGBoost, Lasso</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>GAM</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>playground-series-s3e9</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Regression with a Tabular Concrete Strength Dataset</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>765</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2023-05-15</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M31" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" t="n">
+        <v>3</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>blending</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>Nonlinear features for linear regression (from partial dependence plots); feature selection by CV; target encoding of AgeInDays (treated as categorical)</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>LightGBM, GradientBoosting, RandomForest, LinearRegression</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>playground-series-s3e8</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Regression with a Tabular Gemstone Price Dataset</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>734</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2023-04-30</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M32" t="n">
+        <v>2</v>
+      </c>
+      <c r="N32" t="n">
+        <v>2</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>ordinal</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>Ordinal encoding of gemstone quality categoricals; aspect ratio features; carat x aspect ratio interaction; encoding methodology comparison via CV</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, Ridge, NN</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>playground-series-s3e6</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Regression with a Tabular Paris Housing Price Dataset</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>703</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2023-04-15</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>3</v>
+      </c>
+      <c r="N33" t="n">
+        <v>2</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>Permutation importance for feature selection (per model separately)</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>XGBoost, CatBoost, RandomForest, LightGBM</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>playground-series-s3e1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Regression with a Tabular California Housing Dataset</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>689</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>1</v>
+      </c>
+      <c r="N34" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>kfold</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>Coordinate-based geographic features (from public notebook)</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost, RandomForest, NN</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>playground-series-s3e7</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Binary Classification with a Tabular Reservation Cancellation Dataset</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>678</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2023-04-30</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M35" t="n">
+        <v>1</v>
+      </c>
+      <c r="N35" t="n">
+        <v>2</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>OHE</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>stratified_kfold</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>blending</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>Categorical feature identification; OHE vs native encoding comparison; duplicate/leakage exploitation (opposite label assignment; predict 0.5 for test duplicates); adversarial validation to filter original dataset; removal of train duplicates with test counterparts</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>concat_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>playground-series-s3e3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Binary Classification with a Tabular Employee Attrition Dataset</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>665</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2023-02-28</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>1</v>
+      </c>
+      <c r="N36" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>Domain-driven risk flags (age&lt;34; hourly rate&lt;60; distance&gt;=20; tenure&lt;4 years; job hopper); composite AttritionRisk score; MonthlyIncome/Age ratio; AverageTenure (TotalWorkingYears/NumCompaniesWorked)</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM, CatBoost</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>not_described</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>not_described</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Code-check pass: add code_url and fill fields for 3 entries
- s3e8: code_url set to craigmthomas/play-s3e8-eda-models (already pulled)
- icr: code_url set to room722/icr-adv-model; filled missing_data_strategy,
  encoding_strategy, scaling, cv_strategy, ensemble_method, original_data_usage
  from notebook scan (corrected median assumption to sentinel fill)
- s3e7, s3e13, s3e17, s3e1: confirmed existing coding correct; no code published
Pull notebook for icr and s5e3; add private/ to .gitignore

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kaggle_meta_analysis.xlsx
+++ b/data/kaggle_meta_analysis.xlsx
@@ -738,14 +738,19 @@
           <t>https://www.kaggle.com/competitions/icr-identify-age-related-conditions/discussion?sortBy=voteCount</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>https://www.kaggle.com/room722/icr-adv-model</t>
+        </is>
+      </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>imputation</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>label_encoding</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -755,7 +760,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -765,7 +770,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>repeated_kfold</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -775,7 +780,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>mean_blend</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -800,7 +805,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -1069,6 +1074,11 @@
           <t>https://www.kaggle.com/competitions/playground-series-s5e3/discussion?sortBy=voteCount</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>https://www.kaggle.com/code/cdeotte/rapids-svc-w-feature-engineering-lb-0-856</t>
+        </is>
+      </c>
       <c r="T4" t="inlineStr">
         <is>
           <t>not_described</t>
@@ -1076,7 +1086,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -1086,7 +1096,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -1111,7 +1121,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>No FE; original data added as new columns via target mapping (merge_columns approach)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -1131,7 +1141,7 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>merge_columns</t>
+          <t>concat_rows;merge_columns</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
@@ -3235,7 +3245,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -3260,7 +3270,7 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>stratified_kfold</t>
+          <t>repeated_stratified_kfold</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -3290,7 +3300,7 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>concat_rows; merge_columns</t>
+          <t>concat_rows;merge_columns</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
@@ -3887,7 +3897,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -3937,7 +3947,7 @@
       </c>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>optuna</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -4371,12 +4381,12 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>one_hot_encoding</t>
+          <t>not_described</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -4411,7 +4421,7 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>Piecewise linear encoding (PLE) for continuous features; embedding layers for categorical features (edema, stage)</t>
+          <t>Piecewise linear encoding (PLE) for continuous features; embedding layers for categorical features (edema, stage); value rounding for GBT features</t>
         </is>
       </c>
       <c r="AC24" t="inlineStr">
@@ -5666,6 +5676,11 @@
       <c r="R32" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/competitions/playground-series-s3e8/writeups/craig-thomas-2nd-place-solution</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://www.kaggle.com/code/craigmthomas/play-s3e8-eda-models</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">

</xml_diff>

<commit_message>
Phase 3 complete: EDA notebook, contradiction audit, Results section
- Build notebooks/01_eda.ipynb (7 figures, 9 sections); retire build_bar_plots.py
  and 4 stale presentation plots
- Contradiction audit (scripts/_audit_contradictions.py): reduced 24 flags to 14
  across 12 entries; 8 Excel corrections applied (scripts/_apply_fixes.py)
  including 3 cardinality fixes, 2 feature_type_dominant fixes, 1 cv_strategy
  fix, 1 scaling fix, and clarification of has_categorical for s3e6/s5e5
- Fix methodology section: separator char | → ;, fill rate numbers updated
  (missing_data_strategy 53→16%, scaling 60→27%), limitation reframed
- Write Section 4 Results (all 7 subsections): model/ensemble/CV/encoding
  frequency analysis, cross-tabulations, statistical validation, unexpected
  findings (GBM+scaling, regression+stratified CV, NN in categorical entries)
- Regenerate all 7 EDA figures with corrected data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kaggle_meta_analysis.xlsx
+++ b/data/kaggle_meta_analysis.xlsx
@@ -714,7 +714,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -1221,10 +1221,8 @@
           <t>numeric</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
+      <c r="N5" t="b">
+        <v>0</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1580,7 +1578,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -2415,7 +2413,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -2776,7 +2774,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>stratified_kfold</t>
+          <t>kfold</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -2919,12 +2917,12 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>target_encoding</t>
+          <t>not_described</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -4060,7 +4058,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -4223,7 +4221,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -4676,7 +4674,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -4702,7 +4700,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -4932,7 +4930,7 @@
         <v>360336</v>
       </c>
       <c r="AI27" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
@@ -5023,7 +5021,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -5088,9 +5086,6 @@
       </c>
       <c r="AH28" t="n">
         <v>707</v>
-      </c>
-      <c r="AI28" t="n">
-        <v>11</v>
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
@@ -5527,7 +5522,7 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>target_encoding</t>
+          <t>not_described</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
@@ -5685,7 +5680,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>imputation</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -5817,13 +5812,11 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="N33" t="b">
+        <v>1</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -5848,7 +5841,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>imputation</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -5913,9 +5906,6 @@
       </c>
       <c r="AH33" t="n">
         <v>22730</v>
-      </c>
-      <c r="AI33" t="n">
-        <v>0</v>
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
@@ -6230,9 +6220,6 @@
       <c r="AH35" t="n">
         <v>42100</v>
       </c>
-      <c r="AI35" t="n">
-        <v>0</v>
-      </c>
       <c r="AJ35" t="inlineStr">
         <is>
           <t>Area Under Receiver Operating Characteristic Curve</t>
@@ -6342,7 +6329,7 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>not_described</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
@@ -7145,7 +7132,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -7467,7 +7454,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -7628,7 +7615,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -7789,7 +7776,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -7950,7 +7937,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>none</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">

</xml_diff>

<commit_message>
Revert two bad fixes caused by _scan_notebook.py hardcoded path bug
_scan_notebook.py had a hardcoded path to s3e1's notebook; all scan
calls in the previous commit read that file regardless of the argument
passed, producing false "no StandardScaler / no StratifiedKFold" results.

Reverts:
- s3e3 scaling: not_described → standard (notebook Cell 25 confirms
  StandardScaler().fit_transform() is used on the full feature matrix)
- s4e9 cv_strategy: kfold → stratified_kfold (notebook Cell 86 confirms
  StratifiedKFold is used for the regression task with target binning)

Consequent corrections in research_report.md Section 4:
- stratified_kfold count: 18 → 19 (49%)
- kfold count: 11 → 10 (26%)
- binary classification using stratified KFold: 16 (76%) → 14 (67%)
- GBM+scaling count: 9 → 7 (21% of GBM entries)

Re-regenerated all EDA figures from corrected data.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kaggle_meta_analysis.xlsx
+++ b/data/kaggle_meta_analysis.xlsx
@@ -2774,7 +2774,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>kfold</t>
+          <t>stratified_kfold</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>not_described</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">

</xml_diff>

<commit_message>
Add Pass 2 'Paradigm & Attribution' sheet + build script + journal note
Adds a second sheet to kaggle_meta_analysis.xlsx capturing what the
re-evaluation surfaced that the Pass 1 schema can't represent: paradigm,
origination score (0-3), attribution (cited members, public-notebook forks,
academic citations, canonized-technique uses), author centrality, notable
commenters, and a 200-char unique-edge per winner. 45 rows joined on
(competition_ref, finish_rank). Codebook extended with 15 entries.

Build is idempotent via scripts/build_pass2_sheet.py (re-creates sheet on
each run from the dict-list of row data). Session log updated to record
the pivot away from flowchart deliverable toward descriptive
characterization framing.

Key finding the sheet surfaced: no entries at origination_score=0 (pure
fork) — even the most fork-heavy wins added a meaningful tweak.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kaggle_meta_analysis.xlsx
+++ b/data/kaggle_meta_analysis.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Competition Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Codebook" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Example (icr)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Paradigm &amp; Attribution" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +37,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +61,12 @@
         <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDDDDD"/>
+        <bgColor rgb="00DDDDDD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -69,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -77,6 +88,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8031,7 +8052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8335,6 +8356,193 @@
       <c r="B25" t="inlineStr">
         <is>
           <t>not_used | concat_rows | merge_columns | fold_addition | not_described</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>--- Pass 2 (Paradigm &amp; Attribution sheet) ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>paradigm</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>ensemble-stacking | single-model-FE | lookup-exploit | problem-fit-NN | community-template-tweak | mixed. Primary winning paradigm per per-writeup re-evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>lookup_exploit_subtype</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>identity | inversion | distance-via-generator-flaw | exact-solution-feature | none. Only meaningful when paradigm = lookup-exploit; otherwise 'none'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>lookup_material_present</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>TRUE | FALSE. TRUE if lookup-able material (exact-match, snap, KDTree, original target lookup, etc.) appeared anywhere in the solution, independent of primary paradigm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>origination_score</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>0-3 ordinal. 0=pure fork; 1=fork+small tweak; 2=significant original work on top of community foundation; 3=mostly original (pipeline+FE+models+ensemble all from winner).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>cited_community_members</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Semicolon-separated Kaggle handles named in the writeup as technique/notebook/discussion sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>n_cited_members</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Count derived from cited_community_members.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>forked_from_public_notebook</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>TRUE | FALSE. TRUE if the winning pipeline is built on a single forked public notebook as its base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>academic_papers_cited</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Semicolon-separated short labels (e.g. 'TFT (1912.09363)', 'PLE (2203.05556)').</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>uses_canonized_technique</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Semicolon-separated from {HC, brute-force-FE, Ridge-as-stacker, RAPIDS-XGB, AG-as-ensembler, target-encoding-stack, LAD-as-stacker, original-as-columns, MLP-stacker, DAE-as-base-encoder, pseudo-labeling, adversarial-validation}. Excluded: Optuna, OOF-stacking-generic, GroupKFold, standard model families.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>author_surprise_flag</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>TRUE | FALSE. TRUE if writeup contains explicit 'didn't expect / how on earth / unexpected' framing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>author_recurring_in_set</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>TRUE | FALSE. TRUE if author appears in &gt;1 row of this set (winner or cited source).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>author_appearance_count</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Total appearances of author across set (wins + citations).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>notable_commenters</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Semicolon-separated handles for commenters who are EITHER a Kaggle Grandmaster OR appear elsewhere in our set as winner/cited-source/recurring-author.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>winner_unique_edge</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>One-line (&lt;=200 chars) description of the single thing distinguishing the winner from the public template / runner-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>reeval_doc</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Relative path to per-writeup re-evaluation doc.</t>
         </is>
       </c>
     </row>
@@ -8596,4 +8804,3602 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>competition_ref</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>finish_rank</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>paradigm</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>lookup_exploit_subtype</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>lookup_material_present</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>origination_score</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>cited_community_members</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>n_cited_members</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>forked_from_public_notebook</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>academic_papers_cited</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>uses_canonized_technique</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>author_surprise_flag</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>author_recurring_in_set</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>author_appearance_count</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>notable_commenters</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t>winner_unique_edge</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>reeval_doc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>icr-identify-age-related-conditions</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>room722</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>problem-fit-NN</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>SAMUEL/muelsamu</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>TFT (1912.09363)</t>
+        </is>
+      </c>
+      <c r="L2" s="8" t="inlineStr"/>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N2" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte;cpmpml;ravi20076</t>
+        </is>
+      </c>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t>NN-only at 617 rows via Variable Selection Network + dropout 0.75 + 10x10-30 repeated CV + multi-label CV + probability reweighting</t>
+        </is>
+      </c>
+      <c r="R2" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/icr_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e7</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>ravi20076+arunklenin (Cross Sellers)</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>rzatemizel;uryednap;tilii7;optimistix</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr"/>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>brute-force-FE;target-encoding-stack</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>tilii7;optimistix</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>3-stage stacking with XGB final stacker; 78 weak learners; 12-version feature store; component models on data subsets; target reversal post-processing</t>
+        </is>
+      </c>
+      <c r="R3" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e7_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e3</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="8" t="inlineStr"/>
+      <c r="I4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr"/>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>RAPIDS-XGB;original-as-columns</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O4" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr"/>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>Tiny-data playbook: no FE (curse of dimensionality), equal-weight mean blend of 3 models (XGB+TabPFN+RAPIDS SVC poly), Group K Fold by year</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e3_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e5</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="8" t="inlineStr"/>
+      <c r="I5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr"/>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>HC;RAPIDS-XGB;target-encoding-stack</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>mahog</t>
+        </is>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>GPU Hill Climbing canonization here; 7-model HC ensemble; residual modeling chain (LR-&gt;NN-&gt;XGB); groupby z-score features (26)</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e5_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e12</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>wind1234it</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>masayakawamata;daylighth;laureanoarcanio;tilii7;mikhailnaumov;siukeitin</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr"/>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>HC;Ridge-as-stacker;original-as-columns</t>
+        </is>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>masayakawamata;tilii7</t>
+        </is>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>Post-cutoff CV (cutoff_id=678260) + HC with negative weights + Ridge stacker on rank-transformed top-36; ~100 base OOFs; anti-greedy submission</t>
+        </is>
+      </c>
+      <c r="R6" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e12_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e10</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>tilii7</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>masayakawamata;cdeotte;siukeitin;optimistix;mikhailnaumov;mahoganybuttstrings</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr"/>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>HC;MLP-stacker;DAE-as-base-encoder</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte;masayakawamata</t>
+        </is>
+      </c>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t>11 genetic programming features added at ENSEMBLE stage (not base); Lasso used to reverse-engineer generator formula; Keras NN + CatBoost intermediate stackers</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e10_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e10</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>omidbaghchehsaraei</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>paddykb;siukeitin</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr"/>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>HC</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>ravaghi;siukeitin</t>
+        </is>
+      </c>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>HC (hillclimbers library) over 21-24 models including paddykb's all-as-categorical port; anti-greedy submission (lower public LB, higher CV)</t>
+        </is>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e10_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e11</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>mahoganybuttstrings</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>masayakawamata;cdeotte;yekenot;yeoyunsianggeremie;jklol86;mikhailnaumov</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr"/>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>HC;Ridge-as-stacker;target-encoding-stack</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte;tilii7</t>
+        </is>
+      </c>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t>Diversity-without-tuning: 23 model families with default HP + digit interaction combinatorics + TE with alternative targets (employment_status, debt_to_income)</t>
+        </is>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e11_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e1</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>iqbalsyahakbar</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>arunklenin;aspillai;paddykb</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr"/>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>Ridge-as-stacker;target-encoding-stack</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>paddykb;aspillai</t>
+        </is>
+      </c>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t>TF-IDF+SVD on text-like Surname then encode SVD components via CatBoost (double-layer FE); 30-fold CV for submission; CatBoost-encoder order-sensitivity</t>
+        </is>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e1_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e2</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>single-model-FE</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>jordanbarker</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr"/>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>brute-force-FE;target-encoding-stack;RAPIDS-XGB;original-as-columns</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr"/>
+      <c r="Q11" s="8" t="inlineStr">
+        <is>
+          <t>Single XGB with 500 engineered features on 4M rows; histogram-binned groupby aggs (cdeotte invention); NaN base-2 encoding; nested-fold target-aware FE</t>
+        </is>
+      </c>
+      <c r="R11" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e2_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e8</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>mahoganybuttstrings</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte;omidbaghchehsaraei;yekenot;itasps;siukeitin;tilii7</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr"/>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>HC;target-encoding-stack</t>
+        </is>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte;tilii7</t>
+        </is>
+      </c>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t>CatBoost as final stacker (beat Ridge by 0.00010 on private) in head-to-head 4-stacker test; 13 model architectures; TE on bigrams using comp + original targets</t>
+        </is>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e8_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e4</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>greysky</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>single-model-FE</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" s="8" t="inlineStr"/>
+      <c r="I13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr"/>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>target-encoding-stack</t>
+        </is>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte</t>
+        </is>
+      </c>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>Single LightGBM minimalist: 1552 features via 6-way TE combinatorics + descriptive stats; no CV, no ensemble, no HP tuning; Kaggle parallel-notebook experimentation</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e4_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e9</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>martinapreusse</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>yekenot;siukeitin;tilii7;roberthatch;noodl35;cdeotte</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr"/>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>MLP-stacker;Ridge-as-stacker</t>
+        </is>
+      </c>
+      <c r="M14" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte</t>
+        </is>
+      </c>
+      <c r="Q14" s="8" t="inlineStr">
+        <is>
+          <t>Last-day fork of yekenot's DeepTables NN starter + added 4 OOFs as features = NN-as-stacker won; outlier classification via IQR; median TE</t>
+        </is>
+      </c>
+      <c r="R14" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e9_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e5</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>adaubas (aldparis)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>mfmfmf3;igorvolianiuk;siukeitin;act18l;ambrosm;tilii7</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr"/>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Ridge-as-stacker</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>innixma;tilii7;ambrosm</t>
+        </is>
+      </c>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>EDA-driven discovery: dataset is Poisson sum -&gt; row-wise stats FE; Ridge with negative weights (positive=False); only 2 submissions in 13 days (trust-CV)</t>
+        </is>
+      </c>
+      <c r="R15" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e5_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e11</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>ravaghi</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>optimistix;tilii7</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr"/>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>AG-as-ensembler</t>
+        </is>
+      </c>
+      <c r="M16" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>optimistix;tilii7</t>
+        </is>
+      </c>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>AutoGluon as final stacker (chosen over HC/Ridge/LR head-to-head); 24 models selected from 69; 4 data pipelines for diversity; anti-greedy submission</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e11_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e6</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>bizen250;ayushchandramaurya;elainedazzio;ricopue</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr"/>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>HC;target-encoding-stack;RAPIDS-XGB;original-as-columns;pseudo-labeling</t>
+        </is>
+      </c>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>mahog</t>
+        </is>
+      </c>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>Original-as-columns + cuDF TE at scale: 162 combos x 7 binary targets x 2 datasets = 2268 features; boosting over LR residuals; multi-seed averaging tuned to MAP@K</t>
+        </is>
+      </c>
+      <c r="R17" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e6_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e8</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>optimistix</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>exact-solution-feature</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>ambrosm;siukeitin;nischaydnk;gauravduttakiit;rzatemizel;ravaghi;oscarm524;ravi20076;tilii7;roberthatch;omidbaghchehsaraei;trupologhelper;arunklenin;carlmcbrideellis</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr"/>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>HC;AG-as-ensembler;Ridge-as-stacker</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O18" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>ravaghi;tilii7;ravi20076</t>
+        </is>
+      </c>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t>Confident-disagreement-overwriting (&gt;0.99 threshold inserts) + 72 OOFs into AutoGluon-as-ensembler; three independent stacker paths converged at 0.98535</t>
+        </is>
+      </c>
+      <c r="R18" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e8_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e12</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>single-model-FE</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" s="8" t="inlineStr"/>
+      <c r="I19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr"/>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>brute-force-FE;target-encoding-stack;RAPIDS-XGB</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P19" s="8" t="inlineStr"/>
+      <c r="Q19" s="8" t="inlineStr">
+        <is>
+          <t>GPU brute-force search of 145K+ categorical combinations -&gt; kept 170 that moved CV; explicit FE-effectiveness conditioning as strategy axis</t>
+        </is>
+      </c>
+      <c r="R19" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e12_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e3</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>yunqicao (Moonlit)</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>community-template-tweak</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>noepinefrin;arunklenin;cyrilbourgeois;thomasmeiner;ankurgarg04;lucamassaron;arnogils</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr"/>
+      <c r="L20" s="8" t="inlineStr"/>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P20" s="8" t="inlineStr">
+        <is>
+          <t>arunklenin</t>
+        </is>
+      </c>
+      <c r="Q20" s="8" t="inlineStr">
+        <is>
+          <t>Fork-heavy first-time competitor: 3 OOF ensembles (1 own + 2 public-notebook replications) + Nelder-Mead weights; public-notebook blend alone scores top-10</t>
+        </is>
+      </c>
+      <c r="R20" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e3_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e24</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>ravi20076</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>arunklenin;cv13j0;oscarm524;paddykb</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr"/>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>brute-force-FE</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O21" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>paddykb;oscarm524</t>
+        </is>
+      </c>
+      <c r="Q21" s="8" t="inlineStr">
+        <is>
+          <t>Brute-force FE search at Dec 2023 (predates cdeotte by 12 months, sourced from arunklenin); 8 model families incl TabNet+GAM; 10x1 vs 10x3 CV comparison</t>
+        </is>
+      </c>
+      <c r="R21" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e24_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e23</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>oscarm524</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>ambrosm;sauravpandey11</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr"/>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>HC</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>ambrosm</t>
+        </is>
+      </c>
+      <c r="Q22" s="8" t="inlineStr">
+        <is>
+          <t>HC ensemble of 8 models at Nov 2023 (predates cdeotte canonization by 18 months); log-transform on all features; Nystrom LogisticRegression</t>
+        </is>
+      </c>
+      <c r="R22" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e23_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e14</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>sergiosaharovskiy</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>lookup-exploit</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>zhukovoleksiy;paddykb;yzokulu;tetsutani;adaubas;mattop</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K23" s="8" t="inlineStr"/>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>LAD-as-stacker</t>
+        </is>
+      </c>
+      <c r="M23" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N23" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>adaubas;paddykb</t>
+        </is>
+      </c>
+      <c r="Q23" s="8" t="inlineStr">
+        <is>
+          <t>Match test rows to original dataset by (fruitset, fruitmass) keys; assign exact original yield values (776 unique yields, 2073 test rows); largest 1-2 gap (0.657 MAE)</t>
+        </is>
+      </c>
+      <c r="R23" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e14_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e26</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>hardyxu52</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H24" s="8" t="inlineStr"/>
+      <c r="I24" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>PLE (2203.05556)</t>
+        </is>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>MLP-stacker</t>
+        </is>
+      </c>
+      <c r="M24" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N24" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O24" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr"/>
+      <c r="Q24" s="8" t="inlineStr">
+        <is>
+          <t>PLE for continuous features in NN; NN-as-final-stacker with per-class probability weights + cross-prediction weight calculation; 10 Optuna sets averaged per GBDT</t>
+        </is>
+      </c>
+      <c r="R24" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e26_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e16</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>ravi20076</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>pandeyg0811;inversion</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr"/>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>LAD-as-stacker</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N25" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O25" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="P25" s="8" t="inlineStr"/>
+      <c r="Q25" s="8" t="inlineStr">
+        <is>
+          <t>Generator-driven data augmentation (run official generator notebook with varied params); domain features (meat yield, pseudo BMI); feature-subset diversity per model</t>
+        </is>
+      </c>
+      <c r="R25" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e16_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e17</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>mathurinache (ISoft)</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" s="8" t="inlineStr"/>
+      <c r="I26" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K26" s="8" t="inlineStr"/>
+      <c r="L26" s="8" t="inlineStr"/>
+      <c r="M26" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N26" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O26" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P26" s="8" t="inlineStr"/>
+      <c r="Q26" s="8" t="inlineStr">
+        <is>
+          <t>Pure-AutoML stack-of-stacks: 5 AutoML frameworks (Light AutoML, H2O, FLAML, Lazy Classifier, proprietary Statmining) ensembled; 6h on 4 cores 8GB; 10% public ports</t>
+        </is>
+      </c>
+      <c r="R26" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e17_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e11</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>ambrosm</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" s="8" t="inlineStr"/>
+      <c r="I27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="inlineStr"/>
+      <c r="L27" s="8" t="inlineStr">
+        <is>
+          <t>Ridge-as-stacker;target-encoding-stack</t>
+        </is>
+      </c>
+      <c r="M27" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N27" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O27" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P27" s="8" t="inlineStr">
+        <is>
+          <t>sergiosaharovskiy</t>
+        </is>
+      </c>
+      <c r="Q27" s="8" t="inlineStr">
+        <is>
+          <t>Earliest Ridge-as-stacker (Jun 2023); 18-model Zoo + Ridge weights; duplicate-grouping (360K-&gt;3K); PDP-based numerical-as-categorical detection (store_sqft)</t>
+        </is>
+      </c>
+      <c r="R27" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e11_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e13</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>mufathurrohman (Umar)</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>belati;mpwolke</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K28" s="8" t="inlineStr"/>
+      <c r="L28" s="8" t="inlineStr">
+        <is>
+          <t>DAE-as-base-encoder</t>
+        </is>
+      </c>
+      <c r="M28" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N28" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O28" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P28" s="8" t="inlineStr"/>
+      <c r="Q28" s="8" t="inlineStr">
+        <is>
+          <t>First-time competitor: 3-model mean-blend (LGBM + NN + frozen-encoder autoencoder-classifier) at 707 rows; default HP; cites 7-yr-old Porto Seguro autoencoder thread</t>
+        </is>
+      </c>
+      <c r="R28" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e13_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e5</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>rapela (Heitor)</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>single-model-FE</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>paddykb;abhishek;carlmcbrideellis</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K29" s="8" t="inlineStr"/>
+      <c r="L29" s="8" t="inlineStr">
+        <is>
+          <t>RAPIDS-XGB</t>
+        </is>
+      </c>
+      <c r="M29" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N29" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O29" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P29" s="8" t="inlineStr">
+        <is>
+          <t>paddykb</t>
+        </is>
+      </c>
+      <c r="Q29" s="8" t="inlineStr">
+        <is>
+          <t>Earliest single-model winner (Mar 2023): single RAPIDS XGBoost + OptimizedRounder (paddykb) + Optuna + 10-fold CV; chose NOT to use original (CV-driven)</t>
+        </is>
+      </c>
+      <c r="R29" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e5_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e10</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>seascape</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>single-model-FE</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" s="8" t="inlineStr"/>
+      <c r="I30" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K30" s="8" t="inlineStr"/>
+      <c r="L30" s="8" t="inlineStr"/>
+      <c r="M30" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N30" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O30" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P30" s="8" t="inlineStr">
+        <is>
+          <t>paddykb;adaubas</t>
+        </is>
+      </c>
+      <c r="Q30" s="8" t="inlineStr">
+        <is>
+          <t>GAM as PRIMARY model (R .Rmd); XGB+Lasso predictions DEMOTED to input features for GAM; anti-boosting philosophy; reversed stacker hierarchy</t>
+        </is>
+      </c>
+      <c r="R30" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e10_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e9</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>ambrosm</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H31" s="8" t="inlineStr"/>
+      <c r="I31" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K31" s="8" t="inlineStr"/>
+      <c r="L31" s="8" t="inlineStr"/>
+      <c r="M31" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N31" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O31" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P31" s="8" t="inlineStr"/>
+      <c r="Q31" s="8" t="inlineStr">
+        <is>
+          <t>First explicit anti-Optuna stance (manual HP &gt; Optuna); 7-model zoo + mean blend; quantitative trust-CV argument (5407 train vs 721 public LB = coin flip); PDP-based AgeInDays-as-categorical</t>
+        </is>
+      </c>
+      <c r="R31" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e9_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e8</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>craigmthomas</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" s="8" t="inlineStr"/>
+      <c r="I32" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K32" s="8" t="inlineStr"/>
+      <c r="L32" s="8" t="inlineStr">
+        <is>
+          <t>Ridge-as-stacker</t>
+        </is>
+      </c>
+      <c r="M32" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N32" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O32" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P32" s="8" t="inlineStr"/>
+      <c r="Q32" s="8" t="inlineStr">
+        <is>
+          <t>Custom AutoML-like framework: 1,816 total models (1709 L1 + 105 L2 + Ridge stacker); threshold-based first-level selection; lookup-exploit TESTED and rejected (overfit public LB)</t>
+        </is>
+      </c>
+      <c r="R32" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e8_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e6</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>viktortaran</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H33" s="8" t="inlineStr"/>
+      <c r="I33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K33" s="8" t="inlineStr"/>
+      <c r="L33" s="8" t="inlineStr"/>
+      <c r="M33" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N33" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O33" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" s="8" t="inlineStr"/>
+      <c r="Q33" s="8" t="inlineStr">
+        <is>
+          <t>4-GBDT stack with LGBM as metamodel (tree-based stacker, counter to Ridge dominance); permutation importance per model; repeated KFold (5x10)</t>
+        </is>
+      </c>
+      <c r="R33" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e6_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e1</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>kirderf</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>dmitryuarov</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K34" s="8" t="inlineStr">
+        <is>
+          <t>AutoGluon (2003.06505)</t>
+        </is>
+      </c>
+      <c r="L34" s="8" t="inlineStr">
+        <is>
+          <t>AG-as-ensembler</t>
+        </is>
+      </c>
+      <c r="M34" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N34" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P34" s="8" t="inlineStr">
+        <is>
+          <t>innixma</t>
+        </is>
+      </c>
+      <c r="Q34" s="8" t="inlineStr">
+        <is>
+          <t>Earliest AutoGluon-handles-everything win (Jan 2023); ported dmitryuarov's coordinate-based geo FE + AutoGluon = win; author explicit 'pure AutoML wouldn't have won'</t>
+        </is>
+      </c>
+      <c r="R34" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e1_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e7</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>hardyxu52</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>lookup-exploit</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>inversion</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>siukeitin</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K35" s="8" t="inlineStr"/>
+      <c r="L35" s="8" t="inlineStr">
+        <is>
+          <t>adversarial-validation</t>
+        </is>
+      </c>
+      <c r="M35" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N35" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O35" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="P35" s="8" t="inlineStr">
+        <is>
+          <t>siukeitin</t>
+        </is>
+      </c>
+      <c r="Q35" s="8" t="inlineStr">
+        <is>
+          <t>Opposite-label assignment exploit: 716 test rows had train twins with opposite labels; assigned opposite = +0.014 LB; siukeitin's 'predict 0.5 for test duplicates'</t>
+        </is>
+      </c>
+      <c r="R35" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e7_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e3</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>bcruise (Bill Cruise)</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>community-template-tweak</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>khawajaabaidullah</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K36" s="8" t="inlineStr"/>
+      <c r="L36" s="8" t="inlineStr"/>
+      <c r="M36" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N36" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P36" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte</t>
+        </is>
+      </c>
+      <c r="Q36" s="8" t="inlineStr">
+        <is>
+          <t>Forked khawajaabaidullah's 3-GBDT notebook and added 7 domain-driven HR risk-flag features (Age&lt;34, JobHopper, AttritionRisk composite); win was the FE addition</t>
+        </is>
+      </c>
+      <c r="R36" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e3_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s5e7</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>irfanahmad1</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>lookup-exploit</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>exact-solution-feature</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" s="8" t="inlineStr"/>
+      <c r="I37" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K37" s="8" t="inlineStr"/>
+      <c r="L37" s="8" t="inlineStr"/>
+      <c r="M37" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N37" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O37" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P37" s="8" t="inlineStr"/>
+      <c r="Q37" s="8" t="inlineStr">
+        <is>
+          <t>match_p trick: exact-row-join with public original on 7-feature tuple = match_p feature; 5 GBDT variants + Optuna negative-weight blend with threshold tuning</t>
+        </is>
+      </c>
+      <c r="R37" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e7_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s4e4</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>stopwhispering</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>endofnight17j03;inagana;siukeitin</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J38" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K38" s="8" t="inlineStr">
+        <is>
+          <t>OpenFE (Zhang 2022)</t>
+        </is>
+      </c>
+      <c r="L38" s="8" t="inlineStr">
+        <is>
+          <t>adversarial-validation</t>
+        </is>
+      </c>
+      <c r="M38" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N38" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O38" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="P38" s="8" t="inlineStr"/>
+      <c r="Q38" s="8" t="inlineStr">
+        <is>
+          <t>OpenFE academic tool for automated FE + SFS per model family + 49-model Nelder-Mead with negative coefficients (sum=0.997); anti-NN-for-tabular stance; MLOps</t>
+        </is>
+      </c>
+      <c r="R38" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e4_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s3e4</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>olliekemp</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>single-model-FE</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H39" s="8" t="inlineStr"/>
+      <c r="I39" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K39" s="8" t="inlineStr"/>
+      <c r="L39" s="8" t="inlineStr"/>
+      <c r="M39" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N39" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O39" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P39" s="8" t="inlineStr"/>
+      <c r="Q39" s="8" t="inlineStr">
+        <is>
+          <t>Custom CatTune class jointly tunes model params + sampling rate + class weights; 500-CatBoost random-jump pseudo-ensemble via Gaussian HP perturbation; aggregate stats over V cols</t>
+        </is>
+      </c>
+      <c r="R39" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e4_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>tabular-playground-series-feb-2022</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>ambrosm</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>lookup-exploit</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>distance-via-generator-flaw</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>siukeitin</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K40" s="8" t="inlineStr">
+        <is>
+          <t>Knuth AOCP Vol2</t>
+        </is>
+      </c>
+      <c r="L40" s="8" t="inlineStr"/>
+      <c r="M40" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N40" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O40" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P40" s="8" t="inlineStr">
+        <is>
+          <t>siukeitin</t>
+        </is>
+      </c>
+      <c r="Q40" s="8" t="inlineStr">
+        <is>
+          <t>Reverse-engineered np.random.RandomState.choice flaw at source-code level (Knuth Alg K); reverse-transform 286 decamer counts -&gt; 100-element sequence; RadiusNeighborsClassifier wins (single model)</t>
+        </is>
+      </c>
+      <c r="R40" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/tps_feb_2022_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>tabular-playground-series-may-2022</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>ambrosm+pourchot (The Team)</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>problem-fit-NN</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>sudalairajkumar (SRK);cabaxiom;wti200;pourchot</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K41" s="8" t="inlineStr"/>
+      <c r="L41" s="8" t="inlineStr"/>
+      <c r="M41" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N41" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O41" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P41" s="8" t="inlineStr">
+        <is>
+          <t>sudalairajkumar (SRK)</t>
+        </is>
+      </c>
+      <c r="Q41" s="8" t="inlineStr">
+        <is>
+          <t>Architecture-from-data-structure: xgbfir interaction graph has 2 disconnected components -&gt; built NN with 2 branches mirroring graph; LightGBM interaction_constraints tested</t>
+        </is>
+      </c>
+      <c r="R41" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/tps_may_2022_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>tabular-playground-series-jun-2022</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>sebastianvangerwen</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>problem-fit-NN</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>masatomurakawamm;ehekatlact</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J42" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K42" s="8" t="inlineStr">
+        <is>
+          <t>2106.16057;2002.08338</t>
+        </is>
+      </c>
+      <c r="L42" s="8" t="inlineStr">
+        <is>
+          <t>DAE-as-base-encoder</t>
+        </is>
+      </c>
+      <c r="M42" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N42" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O42" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P42" s="8" t="inlineStr"/>
+      <c r="Q42" s="8" t="inlineStr">
+        <is>
+          <t>DAE-for-imputation: task IS missing-value imputation; 7-layer MLP with feature-wise mask embeddings (16-dim); masked MSE loss; conditional output (use pred only at masked positions)</t>
+        </is>
+      </c>
+      <c r="R42" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/tps_jun_2022_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s6e1</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>mahoganybuttstrings</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte;yekenot;omidbaghchehsaraei;siukeitin;masayakawamata;mikhailnaumov</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J43" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K43" s="8" t="inlineStr"/>
+      <c r="L43" s="8" t="inlineStr">
+        <is>
+          <t>Ridge-as-stacker;target-encoding-stack;MLP-stacker</t>
+        </is>
+      </c>
+      <c r="M43" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N43" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O43" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P43" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte;masayakawamata</t>
+        </is>
+      </c>
+      <c r="Q43" s="8" t="inlineStr">
+        <is>
+          <t>Strength-over-diversity inversion (vs mahog's prior diversity-no-tuning); WandB sweeps save ALL trial OOFs (190 total); Ridge + Centered Isotonic at TWO points (per-OOF + post-Ridge)</t>
+        </is>
+      </c>
+      <c r="R43" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e1_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s6e2</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>masayakawamata</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte;tilii7;mahoganybuttstrings;optimistix</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="J44" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K44" s="8" t="inlineStr"/>
+      <c r="L44" s="8" t="inlineStr">
+        <is>
+          <t>HC;Ridge-as-stacker;target-encoding-stack;DAE-as-base-encoder;original-as-columns</t>
+        </is>
+      </c>
+      <c r="M44" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N44" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O44" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P44" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte;tilii7</t>
+        </is>
+      </c>
+      <c r="Q44" s="8" t="inlineStr">
+        <is>
+          <t>Validation discipline headline: chose 0.9557801-CV submission over 0.955865 because CV-LB degraded past 0.95578; would have been 3rd if greedy; 150 OOFs + Optuna selects ~10%</t>
+        </is>
+      </c>
+      <c r="R44" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e2_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s6e3</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>cdeotte</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>ensemble-stacking</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>angelosmar1;azzamradman;badalkrsharma;blamerx;furqonaryadana;greysky;include4eto;johnnyhyland;lightningv08;mahoganybuttstrings;masayakawamata;mikhailnaumov;nalgirayergn;omidbaghchehsaraei;ozermehmet;rawashishsin;siukeitin;tsunamazda;yekenot;yunsuxiaozi;arunklenin</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="J45" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K45" s="8" t="inlineStr"/>
+      <c r="L45" s="8" t="inlineStr">
+        <is>
+          <t>HC;brute-force-FE;Ridge-as-stacker;RAPIDS-XGB;target-encoding-stack;original-as-columns;pseudo-labeling;DAE-as-base-encoder</t>
+        </is>
+      </c>
+      <c r="M45" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N45" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O45" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P45" s="8" t="inlineStr">
+        <is>
+          <t>mahog;masayakawamata</t>
+        </is>
+      </c>
+      <c r="Q45" s="8" t="inlineStr">
+        <is>
+          <t>KGMON Playbook at industrial scale: 850 candidate models from 39 public notebook ports + LLM 'AI Council' (GPT5.4+Gemini3.1+Claude4.6) generating 600K LOC; 4-level stack; snap+KDTree on IBM original</t>
+        </is>
+      </c>
+      <c r="R45" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e3_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>playground-series-s6e4</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>kirill0212 (cstdy)</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>community-template-tweak</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>wguesdon;mahoganybuttstrings;utaazu;yunsuxiaozi;include4eto;yekenot;mikhail_naumov;maria_nadeem;lucas_moraes;rohit;ashish;gnn</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="J46" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K46" s="8" t="inlineStr"/>
+      <c r="L46" s="8" t="inlineStr">
+        <is>
+          <t>Ridge-as-stacker;target-encoding-stack</t>
+        </is>
+      </c>
+      <c r="M46" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="N46" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O46" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P46" s="8" t="inlineStr">
+        <is>
+          <t>mahog</t>
+        </is>
+      </c>
+      <c r="Q46" s="8" t="inlineStr">
+        <is>
+          <t>~90% of OOFs from other Kagglers (wguesdon 30/49% + 24 others); win = meta-architecture: two-binary-classifier reframe of 3-class (Low-vs-Rest + Med-vs-High) + logit LR blend + threshold search</t>
+        </is>
+      </c>
+      <c r="R46" s="8" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e4_rank1.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Split original_data_usage into availability + use_mode columns
Old original_data_usage column conflated two distinct questions
('is an external public original dataset available?' vs 'if so, how is it
used in the solution?'). Re-eval surfaced cases where this hides
meaningful decisions: cdeotte s3e5 chose NOT to use available original
(CV-driven) vs s4e12 had no available original; both coded 'none' previously.

Adds external_original_available (TRUE/FALSE/unknown) and
external_original_use_mode (rows-only/columns-only/both/features-derived/
lookup/available-not-used/unavailable/unknown). 45 rows backfilled from
re-eval docs.

Distribution surfaced:
  available: TRUE 30 / FALSE 12 / unknown 3
  use_mode: rows-only 17, both 8, unavailable 12, available-not-used 2,
            lookup 2, columns-only 1, unknown 3

Old column preserved in-place with deprecation note in Codebook. 90 backfill
entries appended to Corrections Log.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kaggle_meta_analysis.xlsx
+++ b/data/kaggle_meta_analysis.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL46"/>
+  <dimension ref="A1:AN46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -726,6 +726,16 @@
           <t>distribution_shift_type</t>
         </is>
       </c>
+      <c r="AM1" s="12" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="AN1" s="12" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -902,6 +912,16 @@
           <t>covariate</t>
         </is>
       </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1078,6 +1098,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1254,6 +1284,16 @@
           <t>temporal</t>
         </is>
       </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1428,6 +1468,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1599,6 +1649,16 @@
           <t>temporal</t>
         </is>
       </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1770,6 +1830,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1946,6 +2016,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2122,6 +2202,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2298,6 +2388,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2474,6 +2574,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>columns-only</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2650,6 +2760,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2826,6 +2946,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3002,6 +3132,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3173,6 +3313,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>available-not-used</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3349,6 +3499,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3515,6 +3675,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3686,6 +3856,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3862,6 +4042,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4033,6 +4223,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4199,6 +4399,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4370,6 +4580,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4541,6 +4761,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>lookup</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4707,6 +4937,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4878,6 +5118,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5044,6 +5294,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5215,6 +5475,16 @@
           <t>none</t>
         </is>
       </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5378,6 +5648,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN28" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5554,6 +5834,16 @@
           <t>none</t>
         </is>
       </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN29" t="inlineStr">
+        <is>
+          <t>available-not-used</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5730,6 +6020,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM30" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN30" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5901,6 +6201,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6072,6 +6382,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN32" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6241,6 +6561,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN33" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6407,6 +6737,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN34" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6570,6 +6910,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN35" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6741,6 +7091,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM36" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN36" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6915,6 +7275,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM37" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN37" t="inlineStr">
+        <is>
+          <t>lookup</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7089,6 +7459,16 @@
           <t>covariate</t>
         </is>
       </c>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN38" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7263,6 +7643,16 @@
           <t>not-applicable</t>
         </is>
       </c>
+      <c r="AM39" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN39" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7435,6 +7825,16 @@
           <t>covariate</t>
         </is>
       </c>
+      <c r="AM40" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN40" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7604,6 +8004,16 @@
           <t>none</t>
         </is>
       </c>
+      <c r="AM41" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN41" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7773,6 +8183,16 @@
           <t>none</t>
         </is>
       </c>
+      <c r="AM42" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN42" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7942,6 +8362,16 @@
           <t>none</t>
         </is>
       </c>
+      <c r="AM43" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN43" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8111,6 +8541,16 @@
           <t>none</t>
         </is>
       </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN44" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -8280,6 +8720,16 @@
           <t>none</t>
         </is>
       </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN45" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8447,6 +8897,16 @@
       <c r="AL46" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AN46" t="inlineStr">
+        <is>
+          <t>rows-only</t>
         </is>
       </c>
     </row>
@@ -8461,7 +8921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -9032,6 +9492,50 @@
       <c r="B48" s="6" t="inlineStr">
         <is>
           <t>Current values mix availability with use-mode and are scheduled for split. Known issue tracked in 'Data Quality Audit' sheet as proposed-split. Until then: 'none' = neither used nor (in most cases) available; 'yes' = available and used in some unspecified way; explicit modes (concat_rows, merge_columns, both) = use mode is known. s5e10 corrected 2026-05-27 from 'yes' to 'none' (no external original).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>--- Pass 1 split (added 2026-05-27): original_data_usage ---</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>original_data_usage (DEPRECATED)</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>DEPRECATED 2026-05-27. Conflated availability and use mode. Use external_original_available + external_original_use_mode instead. Old values retained for audit trail; new analyses should reference the new columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>TRUE | FALSE | unknown. TRUE if a public external original dataset exists for this competition (regardless of whether the winner used it). 'unknown' when writeup is silent on this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>rows-only | columns-only | both | features-derived | lookup | available-not-used | unavailable | unknown. How the external original is used: rows-only = concatenated as training rows; columns-only = original-as-columns (cdeotte's merge_columns); both = concat + columns; features-derived = aggregated stats from original used as features (e.g. target-mean TE on original); lookup = direct test-to-original key-match or KDTree (the lookup-exploit family); available-not-used = original exists but author deliberately did not use (cv-driven decision); unavailable = no external original exists; unknown = writeup silent.</t>
         </is>
       </c>
     </row>
@@ -14037,7 +14541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14683,6 +15187,3696 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>icr-identify-age-related-conditions</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split.</t>
+        </is>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/icr_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>icr-identify-age-related-conditions</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split.</t>
+        </is>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/icr_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e7</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original + target reversal trick on duplicates.</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e7_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e7</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr"/>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original + target reversal trick on duplicates.</t>
+        </is>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e7_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e3</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr"/>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. cdeotte's deliberate dual-mode use (rows for XGB+TabPFN, columns for SVC).</t>
+        </is>
+      </c>
+      <c r="I19" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e3_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e3</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr"/>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. cdeotte's deliberate dual-mode use (rows for XGB+TabPFN, columns for SVC).</t>
+        </is>
+      </c>
+      <c r="I20" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e3_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e5</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr"/>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Minimally used (concat only); not column-exploited.</t>
+        </is>
+      </c>
+      <c r="I21" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e5_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e5</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr"/>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Minimally used (concat only); not column-exploited.</t>
+        </is>
+      </c>
+      <c r="I22" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e5_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e12</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr"/>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Orig_as_columns base model + concat for others.</t>
+        </is>
+      </c>
+      <c r="I23" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e12_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e12</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr"/>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Orig_as_columns base model + concat for others.</t>
+        </is>
+      </c>
+      <c r="I24" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e12_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e10</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr"/>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H25" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No external original; Lasso reverse-engineered the generator formula from training data (corrected from 'yes' on 2026-05-27).</t>
+        </is>
+      </c>
+      <c r="I25" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e10_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e10</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr"/>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No external original; Lasso reverse-engineered the generator formula from training data (corrected from 'yes' on 2026-05-27).</t>
+        </is>
+      </c>
+      <c r="I26" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e10_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e10</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr"/>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat_rows.</t>
+        </is>
+      </c>
+      <c r="I27" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e10_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e10</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr"/>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H28" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat_rows.</t>
+        </is>
+      </c>
+      <c r="I28" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e10_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e11</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr"/>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public loan dataset concatenated for training rows.</t>
+        </is>
+      </c>
+      <c r="I29" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e11_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e11</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="inlineStr"/>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G30" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H30" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public loan dataset concatenated for training rows.</t>
+        </is>
+      </c>
+      <c r="I30" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e11_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e1</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr"/>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H31" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public bank-churn dataset; CatBoost-encoder-order-sensitivity discovery.</t>
+        </is>
+      </c>
+      <c r="I31" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e1_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e1</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr"/>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H32" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public bank-churn dataset; CatBoost-encoder-order-sensitivity discovery.</t>
+        </is>
+      </c>
+      <c r="I32" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e1_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e2</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr"/>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H33" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. cdeotte 'manufacture suggested retail price' columns-only feature.</t>
+        </is>
+      </c>
+      <c r="I33" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e2_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e2</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr"/>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>columns-only</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H34" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. cdeotte 'manufacture suggested retail price' columns-only feature.</t>
+        </is>
+      </c>
+      <c r="I34" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e2_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e8</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr"/>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H35" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Concat + TE on bigrams using BOTH competition + original targets.</t>
+        </is>
+      </c>
+      <c r="I35" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e8_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e8</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr"/>
+      <c r="F36" s="15" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H36" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Concat + TE on bigrams using BOTH competition + original targets.</t>
+        </is>
+      </c>
+      <c r="I36" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e8_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e4</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr"/>
+      <c r="F37" s="15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H37" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Writeup doesn't explicitly cite external original use.</t>
+        </is>
+      </c>
+      <c r="I37" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e4_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e4</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr"/>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G38" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H38" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Writeup doesn't explicitly cite external original use.</t>
+        </is>
+      </c>
+      <c r="I38" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e4_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e9</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr"/>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H39" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original car-price dataset concat.</t>
+        </is>
+      </c>
+      <c r="I39" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e9_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e9</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr"/>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H40" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original car-price dataset concat.</t>
+        </is>
+      </c>
+      <c r="I40" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e9_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e5</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr"/>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H41" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Original existed but 'completely different from train dataset' — author used for EDA only.</t>
+        </is>
+      </c>
+      <c r="I41" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e5_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e5</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr"/>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>available-not-used</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H42" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Original existed but 'completely different from train dataset' — author used for EDA only.</t>
+        </is>
+      </c>
+      <c r="I42" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e5_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e11</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr"/>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat.</t>
+        </is>
+      </c>
+      <c r="I43" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e11_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e11</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr"/>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H44" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat.</t>
+        </is>
+      </c>
+      <c r="I44" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e11_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e6</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr"/>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H45" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Dual-mode: concat_rows for some models + columns (TE against original) for the 2268-feature monster.</t>
+        </is>
+      </c>
+      <c r="I45" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e6_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e6</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr"/>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H46" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Dual-mode: concat_rows for some models + columns (TE against original) for the 2268-feature monster.</t>
+        </is>
+      </c>
+      <c r="I46" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e6_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e8</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr"/>
+      <c r="F47" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G47" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H47" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Concat + siukeitin's 'exact solution to original' feature (features-derived from original target).</t>
+        </is>
+      </c>
+      <c r="I47" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e8_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e8</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E48" s="15" t="inlineStr"/>
+      <c r="F48" s="15" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="G48" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H48" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Concat + siukeitin's 'exact solution to original' feature (features-derived from original target).</t>
+        </is>
+      </c>
+      <c r="I48" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e8_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e12</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr"/>
+      <c r="F49" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G49" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. First cdeotte writeup without public original.</t>
+        </is>
+      </c>
+      <c r="I49" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e12_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e12</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E50" s="15" t="inlineStr"/>
+      <c r="F50" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G50" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H50" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. First cdeotte writeup without public original.</t>
+        </is>
+      </c>
+      <c r="I50" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e12_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e3</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E51" s="15" t="inlineStr"/>
+      <c r="F51" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G51" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H51" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public UCI steel-plates dataset concat.</t>
+        </is>
+      </c>
+      <c r="I51" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e3_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e3</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E52" s="15" t="inlineStr"/>
+      <c r="F52" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G52" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H52" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public UCI steel-plates dataset concat.</t>
+        </is>
+      </c>
+      <c r="I52" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e3_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e24</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E53" s="15" t="inlineStr"/>
+      <c r="F53" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G53" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H53" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat.</t>
+        </is>
+      </c>
+      <c r="I53" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e24_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e24</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E54" s="15" t="inlineStr"/>
+      <c r="F54" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G54" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H54" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat.</t>
+        </is>
+      </c>
+      <c r="I54" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e24_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e23</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E55" s="15" t="inlineStr"/>
+      <c r="F55" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H55" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original used.</t>
+        </is>
+      </c>
+      <c r="I55" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e23_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e23</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E56" s="15" t="inlineStr"/>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G56" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H56" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original used.</t>
+        </is>
+      </c>
+      <c r="I56" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e23_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e14</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="inlineStr"/>
+      <c r="F57" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G57" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H57" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Lookup exploit: match test rows to original by (fruitset, fruitmass) keys; primary winning mechanism.</t>
+        </is>
+      </c>
+      <c r="I57" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e14_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e14</t>
+        </is>
+      </c>
+      <c r="C58" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E58" s="15" t="inlineStr"/>
+      <c r="F58" s="15" t="inlineStr">
+        <is>
+          <t>lookup</t>
+        </is>
+      </c>
+      <c r="G58" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H58" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Lookup exploit: match test rows to original by (fruitset, fruitmass) keys; primary winning mechanism.</t>
+        </is>
+      </c>
+      <c r="I58" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e14_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e26</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E59" s="15" t="inlineStr"/>
+      <c r="F59" s="15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G59" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H59" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Author didn't disclose external-original use; not_described in Pass 1.</t>
+        </is>
+      </c>
+      <c r="I59" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e26_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e26</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E60" s="15" t="inlineStr"/>
+      <c r="F60" s="15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G60" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H60" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Author didn't disclose external-original use; not_described in Pass 1.</t>
+        </is>
+      </c>
+      <c r="I60" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e26_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e16</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E61" s="15" t="inlineStr"/>
+      <c r="F61" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G61" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H61" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat + generator-driven additional synthetic data.</t>
+        </is>
+      </c>
+      <c r="I61" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e16_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e16</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E62" s="15" t="inlineStr"/>
+      <c r="F62" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G62" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H62" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat + generator-driven additional synthetic data.</t>
+        </is>
+      </c>
+      <c r="I62" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e16_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e17</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E63" s="15" t="inlineStr"/>
+      <c r="F63" s="15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H63" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Writeup minimal (~30 lines); external-original use not described.</t>
+        </is>
+      </c>
+      <c r="I63" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e17_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e17</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E64" s="15" t="inlineStr"/>
+      <c r="F64" s="15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H64" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Writeup minimal (~30 lines); external-original use not described.</t>
+        </is>
+      </c>
+      <c r="I64" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e17_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e11</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E65" s="15" t="inlineStr"/>
+      <c r="F65" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H65" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original media-campaign dataset concat.</t>
+        </is>
+      </c>
+      <c r="I65" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e11_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e11</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="inlineStr"/>
+      <c r="F66" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G66" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H66" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original media-campaign dataset concat.</t>
+        </is>
+      </c>
+      <c r="I66" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e11_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e13</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E67" s="15" t="inlineStr"/>
+      <c r="F67" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G67" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H67" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original used.</t>
+        </is>
+      </c>
+      <c r="I67" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e13_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e13</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E68" s="15" t="inlineStr"/>
+      <c r="F68" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G68" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H68" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original used.</t>
+        </is>
+      </c>
+      <c r="I68" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e13_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e5</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="inlineStr"/>
+      <c r="F69" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G69" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H69" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Original existed but author chose NOT to use (overfit local CV).</t>
+        </is>
+      </c>
+      <c r="I69" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e5_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e5</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="inlineStr"/>
+      <c r="F70" s="15" t="inlineStr">
+        <is>
+          <t>available-not-used</t>
+        </is>
+      </c>
+      <c r="G70" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H70" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Original existed but author chose NOT to use (overfit local CV).</t>
+        </is>
+      </c>
+      <c r="I70" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e5_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e10</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E71" s="15" t="inlineStr"/>
+      <c r="F71" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G71" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H71" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original used.</t>
+        </is>
+      </c>
+      <c r="I71" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e10_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e10</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="inlineStr"/>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H72" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original used.</t>
+        </is>
+      </c>
+      <c r="I72" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e10_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e9</t>
+        </is>
+      </c>
+      <c r="C73" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E73" s="15" t="inlineStr"/>
+      <c r="F73" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G73" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H73" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original used.</t>
+        </is>
+      </c>
+      <c r="I73" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e9_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e9</t>
+        </is>
+      </c>
+      <c r="C74" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E74" s="15" t="inlineStr"/>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G74" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H74" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original used.</t>
+        </is>
+      </c>
+      <c r="I74" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e9_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e8</t>
+        </is>
+      </c>
+      <c r="C75" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E75" s="15" t="inlineStr"/>
+      <c r="F75" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G75" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H75" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public gemstone dataset concat; lookup-exploit TESTED but rejected (overfit public LB).</t>
+        </is>
+      </c>
+      <c r="I75" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e8_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e8</t>
+        </is>
+      </c>
+      <c r="C76" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E76" s="15" t="inlineStr"/>
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H76" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public gemstone dataset concat; lookup-exploit TESTED but rejected (overfit public LB).</t>
+        </is>
+      </c>
+      <c r="I76" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e8_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e6</t>
+        </is>
+      </c>
+      <c r="C77" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D77" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E77" s="15" t="inlineStr"/>
+      <c r="F77" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G77" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H77" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public Paris housing dataset concat.</t>
+        </is>
+      </c>
+      <c r="I77" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e6_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B78" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e6</t>
+        </is>
+      </c>
+      <c r="C78" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D78" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E78" s="15" t="inlineStr"/>
+      <c r="F78" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G78" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H78" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public Paris housing dataset concat.</t>
+        </is>
+      </c>
+      <c r="I78" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e6_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e1</t>
+        </is>
+      </c>
+      <c r="C79" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E79" s="15" t="inlineStr"/>
+      <c r="F79" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G79" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H79" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public California Housing dataset concat.</t>
+        </is>
+      </c>
+      <c r="I79" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e1_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e1</t>
+        </is>
+      </c>
+      <c r="C80" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D80" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E80" s="15" t="inlineStr"/>
+      <c r="F80" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G80" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H80" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public California Housing dataset concat.</t>
+        </is>
+      </c>
+      <c r="I80" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e1_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e7</t>
+        </is>
+      </c>
+      <c r="C81" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E81" s="15" t="inlineStr"/>
+      <c r="F81" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H81" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat + adversarial-validation filter; inversion-lookup exploit.</t>
+        </is>
+      </c>
+      <c r="I81" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e7_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B82" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e7</t>
+        </is>
+      </c>
+      <c r="C82" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E82" s="15" t="inlineStr"/>
+      <c r="F82" s="15" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="G82" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H82" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public original concat + adversarial-validation filter; inversion-lookup exploit.</t>
+        </is>
+      </c>
+      <c r="I82" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e7_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e3</t>
+        </is>
+      </c>
+      <c r="C83" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E83" s="15" t="inlineStr"/>
+      <c r="F83" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G83" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H83" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public IBM HR dataset concat.</t>
+        </is>
+      </c>
+      <c r="I83" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e3_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e3</t>
+        </is>
+      </c>
+      <c r="C84" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E84" s="15" t="inlineStr"/>
+      <c r="F84" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G84" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H84" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public IBM HR dataset concat.</t>
+        </is>
+      </c>
+      <c r="I84" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e3_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B85" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e7</t>
+        </is>
+      </c>
+      <c r="C85" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D85" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E85" s="15" t="inlineStr"/>
+      <c r="F85" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G85" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H85" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. match_p trick: exact-row-join with public original on 7-feature tuple.</t>
+        </is>
+      </c>
+      <c r="I85" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e7_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B86" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s5e7</t>
+        </is>
+      </c>
+      <c r="C86" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E86" s="15" t="inlineStr"/>
+      <c r="F86" s="15" t="inlineStr">
+        <is>
+          <t>lookup</t>
+        </is>
+      </c>
+      <c r="G86" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H86" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. match_p trick: exact-row-join with public original on 7-feature tuple.</t>
+        </is>
+      </c>
+      <c r="I86" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s5e7_rank2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e4</t>
+        </is>
+      </c>
+      <c r="C87" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E87" s="15" t="inlineStr"/>
+      <c r="F87" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G87" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H87" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public UCI Abalone dataset; train-on-original-only-no-validate scheme for distribution-shift handling.</t>
+        </is>
+      </c>
+      <c r="I87" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e4_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B88" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s4e4</t>
+        </is>
+      </c>
+      <c r="C88" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E88" s="15" t="inlineStr"/>
+      <c r="F88" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G88" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H88" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public UCI Abalone dataset; train-on-original-only-no-validate scheme for distribution-shift handling.</t>
+        </is>
+      </c>
+      <c r="I88" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s4e4_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e4</t>
+        </is>
+      </c>
+      <c r="C89" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D89" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E89" s="15" t="inlineStr"/>
+      <c r="F89" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G89" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H89" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No external original used (PCA-anonymized features make exploit-original infeasible).</t>
+        </is>
+      </c>
+      <c r="I89" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e4_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B90" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s3e4</t>
+        </is>
+      </c>
+      <c r="C90" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D90" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E90" s="15" t="inlineStr"/>
+      <c r="F90" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G90" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H90" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No external original used (PCA-anonymized features make exploit-original infeasible).</t>
+        </is>
+      </c>
+      <c r="I90" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s3e4_rank3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="inlineStr">
+        <is>
+          <t>tabular-playground-series-feb-2022</t>
+        </is>
+      </c>
+      <c r="C91" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E91" s="15" t="inlineStr"/>
+      <c r="F91" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G91" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H91" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original; exploit was source-code-level reverse-engineering of np.random.</t>
+        </is>
+      </c>
+      <c r="I91" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/tps_feb_2022_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B92" s="15" t="inlineStr">
+        <is>
+          <t>tabular-playground-series-feb-2022</t>
+        </is>
+      </c>
+      <c r="C92" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D92" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E92" s="15" t="inlineStr"/>
+      <c r="F92" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G92" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H92" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original; exploit was source-code-level reverse-engineering of np.random.</t>
+        </is>
+      </c>
+      <c r="I92" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/tps_feb_2022_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="inlineStr">
+        <is>
+          <t>tabular-playground-series-may-2022</t>
+        </is>
+      </c>
+      <c r="C93" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E93" s="15" t="inlineStr"/>
+      <c r="F93" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G93" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H93" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original.</t>
+        </is>
+      </c>
+      <c r="I93" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/tps_may_2022_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B94" s="15" t="inlineStr">
+        <is>
+          <t>tabular-playground-series-may-2022</t>
+        </is>
+      </c>
+      <c r="C94" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E94" s="15" t="inlineStr"/>
+      <c r="F94" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G94" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H94" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original.</t>
+        </is>
+      </c>
+      <c r="I94" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/tps_may_2022_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="inlineStr">
+        <is>
+          <t>tabular-playground-series-jun-2022</t>
+        </is>
+      </c>
+      <c r="C95" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E95" s="15" t="inlineStr"/>
+      <c r="F95" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G95" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H95" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original.</t>
+        </is>
+      </c>
+      <c r="I95" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/tps_jun_2022_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B96" s="15" t="inlineStr">
+        <is>
+          <t>tabular-playground-series-jun-2022</t>
+        </is>
+      </c>
+      <c r="C96" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E96" s="15" t="inlineStr"/>
+      <c r="F96" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G96" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H96" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No public original.</t>
+        </is>
+      </c>
+      <c r="I96" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/tps_jun_2022_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B97" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s6e1</t>
+        </is>
+      </c>
+      <c r="C97" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D97" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E97" s="15" t="inlineStr"/>
+      <c r="F97" s="15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G97" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H97" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No external dataset used; first of s6 quartet without one.</t>
+        </is>
+      </c>
+      <c r="I97" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e1_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B98" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s6e1</t>
+        </is>
+      </c>
+      <c r="C98" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E98" s="15" t="inlineStr"/>
+      <c r="F98" s="15" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G98" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H98" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. No external dataset used; first of s6 quartet without one.</t>
+        </is>
+      </c>
+      <c r="I98" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e1_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B99" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s6e2</t>
+        </is>
+      </c>
+      <c r="C99" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E99" s="15" t="inlineStr"/>
+      <c r="F99" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G99" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H99" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public heart-disease original + target stats (mean/smoothed/WoE/entropy) as external TE features.</t>
+        </is>
+      </c>
+      <c r="I99" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e2_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B100" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s6e2</t>
+        </is>
+      </c>
+      <c r="C100" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E100" s="15" t="inlineStr"/>
+      <c r="F100" s="15" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="G100" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H100" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. Public heart-disease original + target stats (mean/smoothed/WoE/entropy) as external TE features.</t>
+        </is>
+      </c>
+      <c r="I100" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e2_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B101" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s6e3</t>
+        </is>
+      </c>
+      <c r="C101" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D101" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E101" s="15" t="inlineStr"/>
+      <c r="F101" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G101" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H101" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. IBM Telco Customer Churn (7,032 rows) + snap features + cKDTree nearest-neighbor lookup + PCA/GRP projection fitted on original.</t>
+        </is>
+      </c>
+      <c r="I101" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e3_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B102" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s6e3</t>
+        </is>
+      </c>
+      <c r="C102" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E102" s="15" t="inlineStr"/>
+      <c r="F102" s="15" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="G102" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H102" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. IBM Telco Customer Churn (7,032 rows) + snap features + cKDTree nearest-neighbor lookup + PCA/GRP projection fitted on original.</t>
+        </is>
+      </c>
+      <c r="I102" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e3_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B103" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s6e4</t>
+        </is>
+      </c>
+      <c r="C103" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D103" s="15" t="inlineStr">
+        <is>
+          <t>external_original_available</t>
+        </is>
+      </c>
+      <c r="E103" s="15" t="inlineStr"/>
+      <c r="F103" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G103" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H103" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. External miadul/irrigation-water-requirement-prediction-dataset concatenated.</t>
+        </is>
+      </c>
+      <c r="I103" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e4_rank1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>playground-series-s6e4</t>
+        </is>
+      </c>
+      <c r="C104" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" s="15" t="inlineStr">
+        <is>
+          <t>external_original_use_mode</t>
+        </is>
+      </c>
+      <c r="E104" s="15" t="inlineStr"/>
+      <c r="F104" s="15" t="inlineStr">
+        <is>
+          <t>rows-only</t>
+        </is>
+      </c>
+      <c r="G104" s="15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H104" s="15" t="inlineStr">
+        <is>
+          <t>Backfilled from original_data_usage split. External miadul/irrigation-water-requirement-prediction-dataset concatenated.</t>
+        </is>
+      </c>
+      <c r="I104" s="15" t="inlineStr">
+        <is>
+          <t>analysis/writeup-reevaluation/s6e4_rank1.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>